<commit_message>
Sync prices from July 2026 HAODE list
</commit_message>
<xml_diff>
--- a/data/products-master.xlsx
+++ b/data/products-master.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>70</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -641,7 +641,6 @@
           <t>/haode-web/assets/products/productos-ai/aimb-g5-ai-smart-glasses/main.jpg</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -681,7 +680,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -689,7 +688,6 @@
           <t>/haode-web/assets/products/productos-ai/w630-ai-smart-glasses/main.jpg</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -729,7 +727,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -737,7 +735,6 @@
           <t>/haode-web/assets/products/productos-ai/s1-ai-classic/main.png</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -785,7 +782,6 @@
           <t>/haode-web/assets/products/micas-hd-clear/main.png</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -833,7 +829,6 @@
           <t>/haode-web/assets/products/home-cut-machine/micas-mate.svg</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -881,7 +876,6 @@
           <t>/haode-web/assets/products/home-cut-machine/micas-privacidad.svg</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -929,7 +923,6 @@
           <t>/haode-web/assets/products/cut-machine/x200t/main.jpg</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -964,12 +957,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>650</t>
+          <t>550</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1016,12 +1009,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>650</t>
+          <t>550</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1029,7 +1022,6 @@
           <t>/haode-web/assets/products/samsung-incell/note-10-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1064,12 +1056,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>680</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>670</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1077,7 +1069,6 @@
           <t>/haode-web/assets/products/samsung-incell/note-20-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1112,12 +1103,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1125,7 +1116,6 @@
           <t>/haode-web/assets/products/samsung-incell/note-8/main.jpg</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1160,12 +1150,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1173,7 +1163,6 @@
           <t>/haode-web/assets/products/samsung-incell/note-9/main.jpg</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1208,12 +1197,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>380</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>370</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1260,12 +1249,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>380</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>370</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1312,12 +1301,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>580</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1325,7 +1314,6 @@
           <t>/haode-web/assets/products/samsung-incell/s10e/main.jpg</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1469,7 +1457,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1529,7 +1517,6 @@
           <t>/haode-web/assets/products/samsung-incell/s20-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1577,7 +1564,6 @@
           <t>/haode-web/assets/products/samsung-incell/s21-fe/main.jpg</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1625,7 +1611,6 @@
           <t>/haode-web/assets/products/samsung-incell/s21/main.jpg</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1673,7 +1658,6 @@
           <t>/haode-web/assets/products/samsung-incell/s21-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1708,12 +1692,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>550</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>530</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1721,7 +1705,6 @@
           <t>/haode-web/assets/products/samsung-incell/s21-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1756,12 +1739,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1769,7 +1752,6 @@
           <t>/haode-web/assets/products/samsung-incell/s22/main.jpg</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1804,12 +1786,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>500</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1817,7 +1799,6 @@
           <t>/haode-web/assets/products/samsung-incell/s22-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1852,12 +1833,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>580</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1904,12 +1885,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>650</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>630</t>
+          <t>580</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1917,7 +1898,6 @@
           <t>/haode-web/assets/products/samsung-incell/s23/main.jpg</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -1952,12 +1932,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>650</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>630</t>
+          <t>580</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1965,7 +1945,6 @@
           <t>/haode-web/assets/products/samsung-incell/s23-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2000,12 +1979,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>650</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>630</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2052,12 +2031,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>700</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>680</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2065,7 +2044,6 @@
           <t>/haode-web/assets/products/samsung-incell/s24/main.png</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2100,12 +2078,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>700</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>680</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2113,7 +2091,6 @@
           <t>/haode-web/assets/products/samsung-incell/s24-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2148,12 +2125,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>750</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>950</t>
+          <t>740</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2161,7 +2138,6 @@
           <t>/haode-web/assets/products/samsung-incell/s24-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2196,12 +2172,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>360</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>350</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2209,7 +2185,6 @@
           <t>/haode-web/assets/products/samsung-incell/s8/main.jpg</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2244,12 +2219,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>370</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>360</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2296,12 +2271,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>360</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>350</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2309,7 +2284,6 @@
           <t>/haode-web/assets/products/samsung-incell/s9/main.jpg</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2344,12 +2318,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>370</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>360</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2357,7 +2331,6 @@
           <t>/haode-web/assets/products/samsung-incell/s9-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>价格异常 / 视频缺失</t>
@@ -2405,7 +2378,6 @@
           <t>/haode-web/assets/products/samsung-oled/note-10/main.jpg</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2453,7 +2425,6 @@
           <t>/haode-web/assets/products/samsung-oled/note-10-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2501,7 +2472,6 @@
           <t>/haode-web/assets/products/samsung-oled/note-20/main.jpg</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2549,7 +2519,6 @@
           <t>/haode-web/assets/products/samsung-oled/note-20-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -2582,14 +2551,11 @@
           <t>Pantalla para Samsung Note 9</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/note-9/main.jpg</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2622,14 +2588,11 @@
           <t>Pantalla para Samsung S20</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s20/main.jpg</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2714,14 +2677,11 @@
           <t>Pantalla para Samsung S20 Ultra</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s20-ultra/main.jpg</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2754,14 +2714,11 @@
           <t>Pantalla para Samsung S21</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s21/main.jpg</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2794,14 +2751,11 @@
           <t>Pantalla para Samsung S21 Plus</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s21-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2886,14 +2840,11 @@
           <t>Pantalla para Samsung S22 Plus</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s22-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -2978,14 +2929,11 @@
           <t>Pantalla para Samsung S23 Plus</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s23-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -3070,14 +3018,11 @@
           <t>Pantalla para Samsung S24 Plus</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s24-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -3214,14 +3159,11 @@
           <t>Pantalla para Samsung S9 Plus</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/samsung-oled/s9-plus/main.jpg</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>缺平台 / 视频缺失</t>
@@ -3264,8 +3206,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3308,8 +3248,6 @@
           <t>195</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3352,8 +3290,6 @@
           <t>210</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3396,8 +3332,6 @@
           <t>210</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3440,8 +3374,6 @@
           <t>240</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3484,8 +3416,6 @@
           <t>220</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3528,8 +3458,6 @@
           <t>245</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3572,8 +3500,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3616,8 +3542,6 @@
           <t>290</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3660,8 +3584,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3704,8 +3626,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3748,8 +3668,6 @@
           <t>290</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3792,8 +3710,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3836,8 +3752,6 @@
           <t>350</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3880,8 +3794,6 @@
           <t>290</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3924,8 +3836,6 @@
           <t>310</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -3968,8 +3878,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4012,8 +3920,6 @@
           <t>380</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4056,8 +3962,6 @@
           <t>380</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4100,8 +4004,6 @@
           <t>730</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4144,8 +4046,6 @@
           <t>280</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4188,8 +4088,6 @@
           <t>380</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4232,8 +4130,6 @@
           <t>680</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4276,8 +4172,6 @@
           <t>950</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4320,8 +4214,6 @@
           <t>2400</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4364,8 +4256,6 @@
           <t>850</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4408,8 +4298,6 @@
           <t>950</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4452,8 +4340,6 @@
           <t>800</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4496,8 +4382,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4540,8 +4424,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4584,8 +4466,6 @@
           <t>175</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4628,8 +4508,6 @@
           <t>190</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -4721,7 +4599,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>190</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -5665,7 +5543,6 @@
           <t>/haode-web/assets/products/iphone-incell/16plus/main.jpg</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5713,7 +5590,6 @@
           <t>/haode-web/assets/products/iphone-incell/16pro/main.jpg</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5761,7 +5637,6 @@
           <t>/haode-web/assets/products/iphone-incell/16promax/main.jpg</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5796,12 +5671,12 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>400</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -5809,7 +5684,6 @@
           <t>/haode-web/assets/products/iphone-incell/16e/main.jpg</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5857,7 +5731,6 @@
           <t>/haode-web/assets/products/iphone-incell/17air/main.jpg</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5905,7 +5778,6 @@
           <t>/haode-web/assets/products/iphone-incell/17/main.jpg</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -5953,7 +5825,6 @@
           <t>/haode-web/assets/products/iphone-incell/17pro/main.jpg</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -6001,7 +5872,6 @@
           <t>/haode-web/assets/products/iphone-incell/17promax/main.jpg</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -6242,14 +6112,11 @@
           <t>Pantalla para iPhone 11</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>185</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6292,8 +6159,6 @@
           <t>590</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6336,8 +6201,6 @@
           <t>640</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6380,8 +6243,6 @@
           <t>830</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6424,8 +6285,6 @@
           <t>720</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6468,8 +6327,6 @@
           <t>780</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6512,8 +6369,6 @@
           <t>850</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6556,8 +6411,6 @@
           <t>950</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
       <c r="J129" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6600,8 +6453,6 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6644,8 +6495,6 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6688,8 +6537,6 @@
           <t>950</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6732,8 +6579,6 @@
           <t>1150</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6776,8 +6621,6 @@
           <t>1250</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6820,8 +6663,6 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
-      <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6864,8 +6705,6 @@
           <t>1950</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6908,8 +6747,6 @@
           <t>720</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
-      <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6952,8 +6789,6 @@
           <t>1450</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
-      <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -6996,8 +6831,6 @@
           <t>180</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
-      <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -7040,8 +6873,6 @@
           <t>570</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
       <c r="J140" t="inlineStr">
         <is>
           <t>ignored_by_product_control=true / historical=true</t>
@@ -7180,12 +7011,12 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>700</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>830</t>
+          <t>680</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -7282,8 +7113,6 @@
           <t>Pantalla para iPhone 12 mini</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/iphone-oled/12mini/main.jpg</t>
@@ -7333,7 +7162,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>700</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -7380,12 +7209,12 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>800</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>780</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -7432,12 +7261,12 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>780</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>760</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -7482,8 +7311,6 @@
           <t>Pantalla para iPhone 13 mini</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/iphone-oled/13mini/main.jpg</t>
@@ -7786,8 +7613,6 @@
           <t>Pantalla para iPhone 15 Plus</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/iphone-oled/15plus/main.jpg</t>
@@ -7882,8 +7707,6 @@
           <t>Pantalla para iPhone 16</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/iphone-oled/16/main.jpg</t>
@@ -7926,8 +7749,6 @@
           <t>Pantalla para iPhone 16 Plus</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
           <t>/haode-web/assets/products/iphone-oled/16plus/main.jpg</t>
@@ -7972,12 +7793,12 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>1400</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>1550</t>
+          <t>1350</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -8037,7 +7858,6 @@
           <t>/haode-web/assets/products/iphone-oled/16promax/main.jpg</t>
         </is>
       </c>
-      <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr">
         <is>
           <t>视频缺失</t>
@@ -8072,12 +7892,12 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1300</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>1450</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -8982,7 +8802,6 @@
           <t>iPhone 12 Pro Max INCELL FHD</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9005,7 +8824,6 @@
           <t>iPhone 14 INCELL FHD</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9028,7 +8846,6 @@
           <t>iPhone 14 Plus INCELL FHD</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9051,7 +8868,6 @@
           <t>iPhone 15 Plus INCELL FHD</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9074,7 +8890,6 @@
           <t>iPhone 13 Pro Max OLED PREMIUM</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9097,7 +8912,6 @@
           <t>Samsung S20 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9120,7 +8934,6 @@
           <t>Samsung S9 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9143,7 +8956,6 @@
           <t>Gafas AI deportivas</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9166,7 +8978,6 @@
           <t>iPhone 16e INCELL FHD</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9189,7 +9000,6 @@
           <t>iPhone 16 Plus INCELL FHD</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9212,7 +9022,6 @@
           <t>iPhone 16 Pro INCELL FHD</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9235,7 +9044,6 @@
           <t>iPhone 16 Pro Max INCELL FHD</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9258,7 +9066,6 @@
           <t>iPhone 17 INCELL FHD</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9281,7 +9088,6 @@
           <t>iPhone 17 Air INCELL FHD</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9304,7 +9110,6 @@
           <t>iPhone 17 Pro INCELL FHD</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9327,7 +9132,6 @@
           <t>iPhone 17 Pro Max INCELL FHD</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9350,7 +9154,6 @@
           <t>iPhone 16 Pro Max SOFT OLED PREMIUM MOVE IC</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9373,7 +9176,6 @@
           <t>Paquete 50 piezas</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9396,7 +9198,6 @@
           <t>Peliculas para corte</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9419,7 +9220,6 @@
           <t>Peliculas privacy</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9442,7 +9242,6 @@
           <t>Gafas AI classic</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9465,7 +9264,6 @@
           <t>Samsung Note 10 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9488,7 +9286,6 @@
           <t>Samsung Note 20 Ultra INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9511,7 +9308,6 @@
           <t>Samsung Note 8 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -9534,7 +9330,6 @@
           <t>Samsung Note 9 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9557,7 +9352,6 @@
           <t>Samsung S20 Ultra INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -9580,7 +9374,6 @@
           <t>Samsung S21 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9603,7 +9396,6 @@
           <t>Samsung S21 Ultra INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9626,7 +9418,6 @@
           <t>Samsung S24 Ultra INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9649,7 +9440,6 @@
           <t>Samsung S8 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9672,7 +9462,6 @@
           <t>Samsung S9 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9695,7 +9484,6 @@
           <t>Samsung S9 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9718,7 +9506,6 @@
           <t>Samsung Note 10 OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -9741,7 +9528,6 @@
           <t>Samsung Note 10 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9764,7 +9550,6 @@
           <t>Samsung Note 20 OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9787,7 +9572,6 @@
           <t>Samsung Note 20 Ultra OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9810,7 +9594,6 @@
           <t>Samsung Note 9 OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -9833,7 +9616,6 @@
           <t>Samsung S20 OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9856,7 +9638,6 @@
           <t>Samsung S20 Ultra OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9879,7 +9660,6 @@
           <t>Samsung S21 OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9902,7 +9682,6 @@
           <t>Samsung S21 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9925,7 +9704,6 @@
           <t>Samsung S22 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9948,7 +9726,6 @@
           <t>Samsung S23 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9971,7 +9748,6 @@
           <t>Samsung S24 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9994,7 +9770,6 @@
           <t>Samsung S9 Plus OLED CON MARCO</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10017,7 +9792,6 @@
           <t>Gafas AI blancas</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10040,7 +9814,6 @@
           <t>X200T</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10063,7 +9836,6 @@
           <t>Samsung S10E INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10086,7 +9858,6 @@
           <t>Samsung S21 FE INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10109,7 +9880,6 @@
           <t>Samsung S21 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10132,7 +9902,6 @@
           <t>Samsung S22 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10155,7 +9924,6 @@
           <t>Samsung S22 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10178,7 +9946,6 @@
           <t>Samsung S23 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10201,7 +9968,6 @@
           <t>Samsung S23 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10224,7 +9990,6 @@
           <t>Samsung S24 INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10247,7 +10012,6 @@
           <t>Samsung S24 Plus INCELL CON MARCO</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>